<commit_message>
feat: land MassCombatPathing (FlowField/AttackSlot/LocalDetour) and warrior pool save
Wire PushMap/Defend agents to scheme B pathing, add 200v200 stress entry, and persist warrior pool with related SPEC/issue updates.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Gravedigger2026/Assets/ConfigTables/Excel/制造_职业配置表_Manufacture_ClassConfig.xlsx
+++ b/Gravedigger2026/Assets/ConfigTables/Excel/制造_职业配置表_Manufacture_ClassConfig.xlsx
@@ -368,12 +368,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -692,7 +698,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -716,16 +722,16 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
@@ -734,90 +740,91 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1167,7 +1174,9 @@
   <dimension ref="A1:H13"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="7"/>
   <cols>
+    <col min="3" max="3" width="17.125" customWidth="1"/>
     <col min="4" max="4" width="10.125" customWidth="1"/>
+    <col min="5" max="5" width="8.875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
@@ -1222,29 +1231,29 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:8">
-      <c r="A3" t="s">
+    <row r="3" s="1" customFormat="1" spans="1:8">
+      <c r="A3" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F3" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="G3" t="s">
+      <c r="G3" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="H3" t="s">
+      <c r="H3" s="1" t="s">
         <v>23</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: PushMap hit FX, MonsterModel_05 assets, and combat presentation polish
Add damage popup/hit flash for PushMap combat, land MonsterModel_05 animations, share projectile combat session, and sync configs/SPEC.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Gravedigger2026/Assets/ConfigTables/Excel/制造_职业配置表_Manufacture_ClassConfig.xlsx
+++ b/Gravedigger2026/Assets/ConfigTables/Excel/制造_职业配置表_Manufacture_ClassConfig.xlsx
@@ -1,37 +1,49 @@
 
-<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Work\Cursor\Gravedigger2026\Gravedigger2026\Gravedigger2026\Assets\ConfigTables\Excel\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <bookViews>
-    <workbookView windowWidth="27945" windowHeight="12255"/>
-  </bookViews>
-  <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-  </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
-</workbook>
+<file path=docProps\app.xml><?xml version="1.0" encoding="utf-8"?>
+<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
+  <Application>Microsoft Excel Compatible / Openpyxl 3.1.5</Application>
+  <HeadingPairs>
+    <vt:vector size="2" baseType="variant">
+      <vt:variant>
+        <vt:lpstr>工作表</vt:lpstr>
+      </vt:variant>
+      <vt:variant>
+        <vt:i4>1</vt:i4>
+      </vt:variant>
+    </vt:vector>
+  </HeadingPairs>
+  <TitlesOfParts>
+    <vt:vector size="1" baseType="lpstr">
+      <vt:lpstr>Sheet1</vt:lpstr>
+    </vt:vector>
+  </TitlesOfParts>
+</Properties>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
+<cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:dcmitype="http://purl.org/dc/dcmitype/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <dc:creator>openpyxl</dc:creator>
+  <cp:lastModifiedBy>王玉栋</cp:lastModifiedBy>
+  <dcterms:created xsi:type="dcterms:W3CDTF">2026-08-06T09:58:00Z</dcterms:created>
+  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-08-07T02:04:45Z</dcterms:modified>
+</cp:coreProperties>
+</file>
+
+<file path=docProps\custom.xml><?xml version="1.0" encoding="utf-8"?>
+<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/custom-properties" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
+  <property fmtid="{D5CDD505-2E9C-101B-9397-08002B2CF9AE}" pid="2" name="ICV">
+    <vt:lpwstr>83B2D260CABF4B8EB01364A4BE897255_12</vt:lpwstr>
+  </property>
+  <property fmtid="{D5CDD505-2E9C-101B-9397-08002B2CF9AE}" pid="3" name="KSOProductBuildVer">
+    <vt:lpwstr>2052-12.1.0.28043</vt:lpwstr>
+  </property>
+  <property fmtid="{D5CDD505-2E9C-101B-9397-08002B2CF9AE}" pid="4" name="CalculationRule">
+    <vt:i4>0</vt:i4>
+  </property>
+</Properties>
+</file>
+
+<file path=xl\sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="57">
   <si>
     <t>职业ID</t>
@@ -115,7 +127,7 @@
     <t>Strength</t>
   </si>
   <si>
-    <t>NormalAttackPrimaryMult_1.5|AttackSpeedBase_0.5|AttackSpeedAgiDiv_60|SkillCdIntDiv_30|SkillCdFloor_0.1</t>
+    <t>NormalAttackPrimaryMult_15|AttackSpeedBase_0.5|AttackSpeedAgiDiv_60|SkillCdIntDiv_30|SkillCdFloor_0.1</t>
   </si>
   <si>
     <t>0.5</t>
@@ -207,7 +219,7 @@
 </sst>
 </file>
 
-<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
   <numFmts count="4">
     <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
@@ -886,7 +898,7 @@
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\theme\theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
@@ -1168,7 +1180,39 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Work\Cursor\Gravedigger2026\Gravedigger2026\Gravedigger2026\Assets\ConfigTables\Excel\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <bookViews>
+    <workbookView windowWidth="27945" windowHeight="12255"/>
+  </bookViews>
+  <sheets>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+  </sheets>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
+</workbook>
+</file>
+
+<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:H13"/>

</xml_diff>

<commit_message>
feat: combat polish through AllyFootCircle, StuckHold, and MonsterModel_06 (v0.75.33)
Land SoftCollision coefficients, edge AttackRange, death knockback, skill-effect config, StuckHold, AllyFootCircle, and MonsterModel_06 art/prefab updates across Defend/PushMap.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Gravedigger2026/Assets/ConfigTables/Excel/制造_职业配置表_Manufacture_ClassConfig.xlsx
+++ b/Gravedigger2026/Assets/ConfigTables/Excel/制造_职业配置表_Manufacture_ClassConfig.xlsx
@@ -1,50 +1,38 @@
 
-<file path=docProps\app.xml><?xml version="1.0" encoding="utf-8"?>
-<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <Application>Microsoft Excel Compatible / Openpyxl 3.1.5</Application>
-  <HeadingPairs>
-    <vt:vector size="2" baseType="variant">
-      <vt:variant>
-        <vt:lpstr>工作表</vt:lpstr>
-      </vt:variant>
-      <vt:variant>
-        <vt:i4>1</vt:i4>
-      </vt:variant>
-    </vt:vector>
-  </HeadingPairs>
-  <TitlesOfParts>
-    <vt:vector size="1" baseType="lpstr">
-      <vt:lpstr>Sheet1</vt:lpstr>
-    </vt:vector>
-  </TitlesOfParts>
-</Properties>
+<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Work\Cursor\Gravedigger2026\Gravedigger2026\Gravedigger2026\Assets\ConfigTables\Excel\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <bookViews>
+    <workbookView windowWidth="27945" windowHeight="12255"/>
+  </bookViews>
+  <sheets>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+  </sheets>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
+</workbook>
 </file>
 
-<file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
-<cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:dcmitype="http://purl.org/dc/dcmitype/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
-  <dc:creator>openpyxl</dc:creator>
-  <cp:lastModifiedBy>王玉栋</cp:lastModifiedBy>
-  <dcterms:created xsi:type="dcterms:W3CDTF">2026-08-06T09:58:00Z</dcterms:created>
-  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-08-07T02:04:45Z</dcterms:modified>
-</cp:coreProperties>
-</file>
-
-<file path=docProps\custom.xml><?xml version="1.0" encoding="utf-8"?>
-<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/custom-properties" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <property fmtid="{D5CDD505-2E9C-101B-9397-08002B2CF9AE}" pid="2" name="ICV">
-    <vt:lpwstr>83B2D260CABF4B8EB01364A4BE897255_12</vt:lpwstr>
-  </property>
-  <property fmtid="{D5CDD505-2E9C-101B-9397-08002B2CF9AE}" pid="3" name="KSOProductBuildVer">
-    <vt:lpwstr>2052-12.1.0.28043</vt:lpwstr>
-  </property>
-  <property fmtid="{D5CDD505-2E9C-101B-9397-08002B2CF9AE}" pid="4" name="CalculationRule">
-    <vt:i4>0</vt:i4>
-  </property>
-</Properties>
-</file>
-
-<file path=xl\sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="57">
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="60">
   <si>
     <t>职业ID</t>
   </si>
@@ -70,6 +58,9 @@
     <t>远程超时</t>
   </si>
   <si>
+    <t>追击移动速度系数</t>
+  </si>
+  <si>
     <t>主键；被 SoulConfig.ClassId 引用</t>
   </si>
   <si>
@@ -94,6 +85,9 @@
     <t>≥0 秒</t>
   </si>
   <si>
+    <t>≥0；仅 GoalKind=AttackSlot 时×移速；缺省1</t>
+  </si>
+  <si>
     <t>ClassId</t>
   </si>
   <si>
@@ -116,6 +110,9 @@
   </si>
   <si>
     <t>RangedTimeoutSeconds</t>
+  </si>
+  <si>
+    <t>ChaseMoveSpeedMult</t>
   </si>
   <si>
     <t>Class_Warrior</t>
@@ -219,7 +216,7 @@
 </sst>
 </file>
 
-<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
   <numFmts count="4">
     <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
@@ -689,148 +686,148 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="4">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="5">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="4">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="6">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="13" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="14" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="15" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="16" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="17" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="18" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="19" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="20" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="22" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="23" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="24" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="25" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="26" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="27" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="28" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="29" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="30" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="31" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="32" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -898,7 +895,7 @@
 </styleSheet>
 </file>
 
-<file path=xl\theme\theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
@@ -1180,50 +1177,18 @@
 </a:theme>
 </file>
 
-<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Work\Cursor\Gravedigger2026\Gravedigger2026\Gravedigger2026\Assets\ConfigTables\Excel\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <bookViews>
-    <workbookView windowWidth="27945" windowHeight="12255"/>
-  </bookViews>
-  <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-  </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
-</workbook>
-</file>
-
-<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:H13"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="7"/>
+  <dimension ref="A1:I13"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="3" max="3" width="17.125" customWidth="1"/>
     <col min="4" max="4" width="10.125" customWidth="1"/>
     <col min="5" max="5" width="8.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:9">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1248,317 +1213,356 @@
       <c r="H1" t="s">
         <v>7</v>
       </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
     </row>
-    <row r="2" spans="1:8">
+    <row r="2" spans="1:9">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H2" t="s">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="I2" t="s">
+        <v>17</v>
       </c>
     </row>
-    <row r="3" s="1" customFormat="1" spans="1:8">
+    <row r="3" s="1" customFormat="1" spans="1:9">
       <c r="A3" s="1" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>23</v>
+        <v>25</v>
+      </c>
+      <c r="I3" t="s">
+        <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:8">
+    <row r="4" spans="1:9">
       <c r="A4" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B4" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="C4" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="D4" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="E4">
         <v>0.3</v>
       </c>
       <c r="F4" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="G4" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="H4" t="s">
-        <v>29</v>
+        <v>32</v>
+      </c>
+      <c r="I4">
+        <v>1.5</v>
       </c>
     </row>
-    <row r="5" spans="1:8">
+    <row r="5" spans="1:9">
       <c r="A5" t="s">
+        <v>33</v>
+      </c>
+      <c r="B5" t="s">
+        <v>34</v>
+      </c>
+      <c r="C5" t="s">
+        <v>35</v>
+      </c>
+      <c r="D5" t="s">
         <v>30</v>
-      </c>
-      <c r="B5" t="s">
-        <v>31</v>
-      </c>
-      <c r="C5" t="s">
-        <v>32</v>
-      </c>
-      <c r="D5" t="s">
-        <v>27</v>
       </c>
       <c r="E5">
         <v>1</v>
       </c>
       <c r="F5" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="G5" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H5" t="s">
-        <v>34</v>
+        <v>37</v>
+      </c>
+      <c r="I5">
+        <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:8">
+    <row r="6" spans="1:9">
       <c r="A6" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="B6" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C6" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="D6" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="E6">
         <v>0.8</v>
       </c>
       <c r="F6" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="G6" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="H6" t="s">
-        <v>34</v>
+        <v>37</v>
+      </c>
+      <c r="I6">
+        <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:8">
+    <row r="7" spans="1:9">
       <c r="A7" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B7" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C7" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="D7" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="E7">
         <v>0.3</v>
       </c>
       <c r="F7" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="G7" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="H7" t="s">
-        <v>29</v>
+        <v>32</v>
+      </c>
+      <c r="I7">
+        <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:8">
+    <row r="8" spans="1:9">
       <c r="A8" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="B8" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="C8" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="D8" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="E8">
         <v>0.3</v>
       </c>
       <c r="F8" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="G8" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="H8" t="s">
-        <v>29</v>
+        <v>32</v>
+      </c>
+      <c r="I8">
+        <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:8">
+    <row r="9" spans="1:9">
       <c r="A9" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="B9" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C9" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="D9" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="E9">
         <v>1.2</v>
       </c>
       <c r="F9" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="G9" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="H9" t="s">
-        <v>46</v>
+        <v>49</v>
+      </c>
+      <c r="I9">
+        <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:8">
+    <row r="10" spans="1:9">
       <c r="A10" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="B10" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="C10" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="D10" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="E10">
         <v>0.3</v>
       </c>
       <c r="F10" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="G10" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="H10" t="s">
-        <v>29</v>
+        <v>32</v>
+      </c>
+      <c r="I10">
+        <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:8">
+    <row r="11" spans="1:9">
       <c r="A11" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="B11" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C11" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="D11" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="E11">
         <v>1.1</v>
       </c>
       <c r="F11" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="G11" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="H11" t="s">
-        <v>34</v>
+        <v>37</v>
+      </c>
+      <c r="I11">
+        <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:8">
+    <row r="12" spans="1:9">
       <c r="A12" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B12" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="C12" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="D12" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="E12">
         <v>0.9</v>
       </c>
       <c r="F12" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="G12" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="H12" t="s">
-        <v>34</v>
+        <v>37</v>
+      </c>
+      <c r="I12">
+        <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:8">
+    <row r="13" spans="1:9">
       <c r="A13" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="B13" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="C13" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="D13" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="E13">
         <v>0.5</v>
       </c>
       <c r="F13" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="G13" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="H13" t="s">
-        <v>29</v>
+        <v>32</v>
+      </c>
+      <c r="I13">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: land GM add-soldier, Mode2 hover tooltip, AttackSlot dual rings, and AllIn1 shader (v0.82.50)
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Gravedigger2026/Assets/ConfigTables/Excel/制造_职业配置表_Manufacture_ClassConfig.xlsx
+++ b/Gravedigger2026/Assets/ConfigTables/Excel/制造_职业配置表_Manufacture_ClassConfig.xlsx
@@ -1038,7 +1038,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:M14"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col width="17.125" customWidth="1" min="3" max="3"/>
@@ -1064,45 +1064,50 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>转职职业</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>等级</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>主属性</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>战斗换算系数</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>攻击距离</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>近战前摇</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>远程弹速</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>远程超时</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>追击移动速度系数</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>制造默认获得技能ID</t>
         </is>
@@ -1121,50 +1126,55 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>CSV 中文：战士|射手|法师|盗贼 → 枚举；空/非法→Unspecified；预留后续魔法书等条件；不参与命名/外观/PrimaryStat/战斗；不烘进实例</t>
+          <t>CSV 中文：战士|射手|法师|刺客 → 枚举；空/非法→Unspecified；预留后续魔法书等条件；不参与命名/外观/PrimaryStat/战斗；不烘进实例</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
+          <t>可选文字；空=无转职目标；本轮仅填表，不驱动玩法</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
           <t>≥0；仅 UI 展示（UI-016 士兵卡职业名下 Lv.{ClassLevel}）；不参与战斗/制造公式；缺/空 → 0</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Strength | Agility | Intelligence</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>键_数值|…；缺键回退全局默认</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>进入攻击态距离</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>≥0 秒；Melee 时用</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>≥0；Ranged 时用</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>≥0 秒</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>≥0；仅 GoalKind=AttackSlot 时×移速；缺省1</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>空=无；SkillId 或 SkillId|SkillId；FK → SkillConfig.SkillId</t>
         </is>
@@ -1188,45 +1198,50 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
+          <t>PromoteClass</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
           <t>ClassLevel</t>
         </is>
       </c>
-      <c r="E3" s="1" t="inlineStr">
+      <c r="F3" s="1" t="inlineStr">
         <is>
           <t>PrimaryStat</t>
         </is>
       </c>
-      <c r="F3" s="1" t="inlineStr">
+      <c r="G3" s="1" t="inlineStr">
         <is>
           <t>CombatConvertCoeffs</t>
         </is>
       </c>
-      <c r="G3" s="1" t="inlineStr">
+      <c r="H3" s="1" t="inlineStr">
         <is>
           <t>AttackRange</t>
         </is>
       </c>
-      <c r="H3" s="1" t="inlineStr">
+      <c r="I3" s="1" t="inlineStr">
         <is>
           <t>MeleeWindupSeconds</t>
         </is>
       </c>
-      <c r="I3" s="1" t="inlineStr">
+      <c r="J3" s="1" t="inlineStr">
         <is>
           <t>RangedProjectileSpeed</t>
         </is>
       </c>
-      <c r="J3" s="1" t="inlineStr">
+      <c r="K3" s="1" t="inlineStr">
         <is>
           <t>RangedTimeoutSeconds</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>ChaseMoveSpeedMult</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>DefaultSkillIds</t>
         </is>
@@ -1248,41 +1263,41 @@
           <t>战士</t>
         </is>
       </c>
-      <c r="D4" t="n">
+      <c r="E4" t="n">
         <v>1</v>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>Strength</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>NormalAttackPrimaryMult_15|AttackSpeedBase_0.5|AttackSpeedAgiDiv_60|SkillCdIntDiv_30|SkillCdFloor_0.1</t>
         </is>
       </c>
-      <c r="G4" t="n">
+      <c r="H4" t="n">
         <v>0.3</v>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>0.5</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="K4" t="n">
+      <c r="L4" t="n">
         <v>2</v>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>Skill_01</t>
         </is>
@@ -1304,38 +1319,38 @@
           <t>射手</t>
         </is>
       </c>
-      <c r="D5" t="n">
+      <c r="E5" t="n">
         <v>1</v>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>Agility</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>NormalAttackPrimaryMult_15|AttackSpeedBase_0.5|AttackSpeedAgiDiv_60|SkillCdIntDiv_30|SkillCdFloor_0.1</t>
         </is>
       </c>
-      <c r="G5" t="n">
+      <c r="H5" t="n">
         <v>1</v>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>0.5</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>13</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="K5" t="n">
+      <c r="L5" t="n">
         <v>0.5</v>
       </c>
     </row>
@@ -1355,38 +1370,38 @@
           <t>法师</t>
         </is>
       </c>
-      <c r="D6" t="n">
+      <c r="E6" t="n">
         <v>1</v>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>Intelligence</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>NormalAttackPrimaryMult_15|AttackSpeedBase_0.5|AttackSpeedAgiDiv_60|SkillCdIntDiv_30|SkillCdFloor_0.1</t>
         </is>
       </c>
-      <c r="G6" t="n">
+      <c r="H6" t="n">
         <v>0.8</v>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>0.5</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>14</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="K6" t="n">
+      <c r="L6" t="n">
         <v>0.5</v>
       </c>
     </row>
@@ -1406,38 +1421,38 @@
           <t>战士</t>
         </is>
       </c>
-      <c r="D7" t="n">
+      <c r="E7" t="n">
         <v>1</v>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>Strength</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>NormalAttackPrimaryMult_15|AttackSpeedBase_0.5|AttackSpeedAgiDiv_60|SkillCdIntDiv_30|SkillCdFloor_0.1</t>
         </is>
       </c>
-      <c r="G7" t="n">
+      <c r="H7" t="n">
         <v>0.3</v>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>0.5</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="K7" t="n">
+      <c r="L7" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1449,46 +1464,46 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>盗贼</t>
+          <t>刺客</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>盗贼</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
+          <t>刺客</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
         <v>1</v>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>Agility</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>NormalAttackPrimaryMult_15|AttackSpeedBase_0.5|AttackSpeedAgiDiv_60|SkillCdIntDiv_30|SkillCdFloor_0.1</t>
         </is>
       </c>
-      <c r="G8" t="n">
+      <c r="H8" t="n">
         <v>0.3</v>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>0.5</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="K8" t="n">
+      <c r="L8" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1508,38 +1523,38 @@
           <t>法师</t>
         </is>
       </c>
-      <c r="D9" t="n">
+      <c r="E9" t="n">
         <v>1</v>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>Intelligence</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>NormalAttackPrimaryMult_15|AttackSpeedBase_0.5|AttackSpeedAgiDiv_60|SkillCdIntDiv_30|SkillCdFloor_0.1</t>
         </is>
       </c>
-      <c r="G9" t="n">
+      <c r="H9" t="n">
         <v>1.2</v>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>0.5</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>17</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K9" t="n">
+      <c r="L9" t="n">
         <v>0.5</v>
       </c>
     </row>
@@ -1559,38 +1574,38 @@
           <t>战士</t>
         </is>
       </c>
-      <c r="D10" t="n">
+      <c r="E10" t="n">
         <v>1</v>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>Strength</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>NormalAttackPrimaryMult_15|AttackSpeedBase_0.5|AttackSpeedAgiDiv_60|SkillCdIntDiv_30|SkillCdFloor_0.1</t>
         </is>
       </c>
-      <c r="G10" t="n">
+      <c r="H10" t="n">
         <v>0.3</v>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>0.5</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="K10" t="n">
+      <c r="L10" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1610,38 +1625,38 @@
           <t>射手</t>
         </is>
       </c>
-      <c r="D11" t="n">
+      <c r="E11" t="n">
         <v>1</v>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>Agility</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>NormalAttackPrimaryMult_15|AttackSpeedBase_0.5|AttackSpeedAgiDiv_60|SkillCdIntDiv_30|SkillCdFloor_0.1</t>
         </is>
       </c>
-      <c r="G11" t="n">
+      <c r="H11" t="n">
         <v>1.1</v>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>0.5</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="K11" t="n">
+      <c r="L11" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1661,38 +1676,38 @@
           <t>法师</t>
         </is>
       </c>
-      <c r="D12" t="n">
+      <c r="E12" t="n">
         <v>1</v>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>Intelligence</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>NormalAttackPrimaryMult_15|AttackSpeedBase_0.5|AttackSpeedAgiDiv_60|SkillCdIntDiv_30|SkillCdFloor_0.1</t>
         </is>
       </c>
-      <c r="G12" t="n">
+      <c r="H12" t="n">
         <v>0.9</v>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>0.5</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="K12" t="n">
+      <c r="L12" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1712,38 +1727,38 @@
           <t>战士</t>
         </is>
       </c>
-      <c r="D13" t="n">
+      <c r="E13" t="n">
         <v>1</v>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>Strength</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>NormalAttackPrimaryMult_15|AttackSpeedBase_0.5|AttackSpeedAgiDiv_60|SkillCdIntDiv_30|SkillCdFloor_0.1</t>
         </is>
       </c>
-      <c r="G13" t="n">
+      <c r="H13" t="n">
         <v>0.5</v>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>0.5</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="J13" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="K13" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="K13" t="n">
+      <c r="L13" t="n">
         <v>1.5</v>
       </c>
     </row>
@@ -1763,38 +1778,38 @@
           <t>战士</t>
         </is>
       </c>
-      <c r="D14" t="n">
+      <c r="E14" t="n">
         <v>1</v>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>Strength</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>NormalAttackPrimaryMult_15|AttackSpeedBase_0.5|AttackSpeedAgiDiv_60|SkillCdIntDiv_30|SkillCdFloor_0.1</t>
         </is>
       </c>
-      <c r="G14" t="n">
+      <c r="H14" t="n">
         <v>0.3</v>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="I14" t="inlineStr">
         <is>
           <t>0.5</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="J14" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="K14" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="K14" t="n">
+      <c r="L14" t="n">
         <v>2.5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: land formation bonds, shop runtime, and skill effect updates
Ship the latest SPEC, config, asset, prefab, and gameplay changes together so the new combat, formation, and shop content stays in sync across data and runtime.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Gravedigger2026/Assets/ConfigTables/Excel/制造_职业配置表_Manufacture_ClassConfig.xlsx
+++ b/Gravedigger2026/Assets/ConfigTables/Excel/制造_职业配置表_Manufacture_ClassConfig.xlsx
@@ -1038,7 +1038,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M14"/>
+  <dimension ref="A1:N14"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col width="17.125" customWidth="1" min="3" max="3"/>
@@ -1104,10 +1104,15 @@
       </c>
       <c r="L1" t="inlineStr">
         <is>
+          <t>基础移速</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
           <t>追击移动速度系数</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>制造默认获得技能ID</t>
         </is>
@@ -1171,10 +1176,15 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
+          <t>&gt;=0；世界单位/秒；士兵 MoveSpeed 维 Base；缺/&lt;=0 -&gt; 3.5</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
           <t>≥0；仅 GoalKind=AttackSlot 时×移速；缺省1</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>空=无；SkillId 或 SkillId|SkillId；FK → SkillConfig.SkillId</t>
         </is>
@@ -1238,10 +1248,15 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
+          <t>BaseMoveSpeed</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
           <t>ChaseMoveSpeedMult</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>DefaultSkillIds</t>
         </is>
@@ -1295,9 +1310,12 @@
         </is>
       </c>
       <c r="L4" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="M4" t="n">
         <v>2</v>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>Skill_01</t>
         </is>
@@ -1351,6 +1369,9 @@
         </is>
       </c>
       <c r="L5" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="M5" t="n">
         <v>0.5</v>
       </c>
     </row>
@@ -1402,6 +1423,9 @@
         </is>
       </c>
       <c r="L6" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="M6" t="n">
         <v>0.5</v>
       </c>
     </row>
@@ -1453,6 +1477,9 @@
         </is>
       </c>
       <c r="L7" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="M7" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1504,6 +1531,9 @@
         </is>
       </c>
       <c r="L8" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="M8" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1555,6 +1585,9 @@
         </is>
       </c>
       <c r="L9" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="M9" t="n">
         <v>0.5</v>
       </c>
     </row>
@@ -1606,6 +1639,9 @@
         </is>
       </c>
       <c r="L10" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="M10" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1657,6 +1693,9 @@
         </is>
       </c>
       <c r="L11" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="M11" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1708,6 +1747,9 @@
         </is>
       </c>
       <c r="L12" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="M12" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1759,6 +1801,9 @@
         </is>
       </c>
       <c r="L13" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="M13" t="n">
         <v>1.5</v>
       </c>
     </row>
@@ -1810,6 +1855,9 @@
         </is>
       </c>
       <c r="L14" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="M14" t="n">
         <v>2.5</v>
       </c>
     </row>

</xml_diff>